<commit_message>
Seguimiento al 30-10: «APK de release» en lugar de «APK firmada», diagramas en StarUML y temas abiertos actualizados
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Roadmap_Proyecto_Barberia_30-10.xlsx
+++ b/Fase 2/Evidencias Proyecto/Roadmap_Proyecto_Barberia_30-10.xlsx
@@ -706,6 +706,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr">
@@ -713,21 +714,33 @@
           <t>Agosto</t>
         </is>
       </c>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="10" t="n"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
       </c>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="10" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
+      <c r="J4" s="9" t="n"/>
+      <c r="K4" s="9" t="n"/>
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="10" t="n"/>
       <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
+      <c r="O4" s="9" t="n"/>
+      <c r="P4" s="9" t="n"/>
+      <c r="Q4" s="10" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1008,7 +1021,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>APK firmada</t>
+          <t>APK de release</t>
         </is>
       </c>
       <c r="O10" s="12" t="inlineStr">
@@ -1105,6 +1118,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="17" t="inlineStr">
         <is>
@@ -1134,8 +1148,8 @@
     <mergeCell ref="I4:M4"/>
     <mergeCell ref="N9:O9"/>
     <mergeCell ref="N11:O11"/>
+    <mergeCell ref="H8:K8"/>
     <mergeCell ref="F6:K6"/>
-    <mergeCell ref="H8:K8"/>
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B6:E6"/>
@@ -1184,6 +1198,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1338,7 +1353,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Despliegue en UAT · APK firmada · limpieza de datos de prueba (JO)</t>
+          <t>Despliegue en UAT · APK de release · limpieza de datos de prueba (JO)</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -1377,6 +1392,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="17" t="inlineStr">
         <is>
@@ -1441,6 +1457,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1635,6 +1652,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1695,6 +1713,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -1729,6 +1748,7 @@
           <t>Atraso de la integración (actividad crítica 1.4.3)</t>
         </is>
       </c>
+      <c r="C10" s="10" t="n"/>
       <c r="D10" s="13" t="inlineStr">
         <is>
           <t>2 × 4 = 8</t>
@@ -1751,6 +1771,7 @@
           <t>Exposición de credenciales o brecha de seguridad</t>
         </is>
       </c>
+      <c r="C11" s="10" t="n"/>
       <c r="D11" s="13" t="inlineStr">
         <is>
           <t>2 × 5 = 10</t>
@@ -1773,6 +1794,7 @@
           <t>Fallas o demoras en la integración con Webpay</t>
         </is>
       </c>
+      <c r="C12" s="10" t="n"/>
       <c r="D12" s="13" t="inlineStr">
         <is>
           <t>2 × 4 = 8</t>
@@ -1795,6 +1817,7 @@
           <t>Pérdida de datos o pausa de la base de datos (plan gratuito de Supabase)</t>
         </is>
       </c>
+      <c r="C13" s="10" t="n"/>
       <c r="D13" s="13" t="inlineStr">
         <is>
           <t>2 × 5 = 10</t>
@@ -1817,6 +1840,7 @@
           <t>Disponibilidad limitada del equipo (2 integrantes)</t>
         </is>
       </c>
+      <c r="C14" s="10" t="n"/>
       <c r="D14" s="13" t="inlineStr">
         <is>
           <t>3 × 3 = 9</t>
@@ -1839,6 +1863,7 @@
           <t>Ventana corta para desplegar y pasar al ambiente UAT (S13–S14)</t>
         </is>
       </c>
+      <c r="C15" s="10" t="n"/>
       <c r="D15" s="13" t="inlineStr">
         <is>
           <t>3 × 3 = 9</t>
@@ -1861,6 +1886,7 @@
           <t>La app Android aún no se prueba en un teléfono real</t>
         </is>
       </c>
+      <c r="C16" s="10" t="n"/>
       <c r="D16" s="13" t="inlineStr">
         <is>
           <t>3 × 3 = 9</t>
@@ -1883,6 +1909,7 @@
           <t>Notificaciones por correo no operativas</t>
         </is>
       </c>
+      <c r="C17" s="10" t="n"/>
       <c r="D17" s="13" t="inlineStr">
         <is>
           <t>3 × 3 = 9</t>
@@ -1905,6 +1932,7 @@
           <t>Las pruebas y el ambiente UAT usan la misma base de datos</t>
         </is>
       </c>
+      <c r="C18" s="10" t="n"/>
       <c r="D18" s="13" t="inlineStr">
         <is>
           <t>3 × 3 = 9</t>
@@ -1968,6 +1996,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2139,7 +2168,7 @@
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>Web publicada en el ambiente UAT (28-10); APK firmada, lista de verificación y pruebas de humo antes del paso</t>
+          <t>Web publicada en el ambiente UAT (28-10); APK de release, lista de verificación y pruebas de humo antes del paso</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
@@ -2176,7 +2205,7 @@
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>APK de prueba lista (28-10); prueba con pago Webpay en un teléfono Android; APK firmada en S13</t>
+          <t>APK de prueba lista (28-10); prueba con pago Webpay en un teléfono Android; APK de release en S13</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">

</xml_diff>